<commit_message>
feat: implement work types and tickets modules with normalization mig… (#26)
* feat: implement work types and tickets modules with normalization migration and planning repository

* fix: linter fix

* fix: another linter fix

* fix: formatter fix

* fix: migration fix

* fix: another migration fix

* feat: normalize work types and tickets with planning eligibility rules and tests

* fix: test fix

* fix: create ticket error

* fix: tests fix

* fix: synthetic datasets generator fix

* fix: formatter fix

* fix: tests fix

* fix: another tests fix
</commit_message>
<xml_diff>
--- a/backend/bruno/fixtures/dataset.xlsx
+++ b/backend/bruno/fixtures/dataset.xlsx
@@ -3512,85 +3512,120 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>work_type_id</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>priority</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>received_at</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>sla_deadline_at</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>required_transport_type</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>service_duration_source</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
           <t>status</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>lifecycle_state</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>visit_window_start</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>visit_window_end</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>planned_start_at</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>planned_end_at</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>estimated_duration_minutes</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>actual_duration_minutes</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>revision</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>execution_cycle</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>actual_started_at</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>actual_completed_at</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>cancel_reason</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>last_event_id</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>created_at</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>updated_at</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
@@ -3620,85 +3655,120 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2026-09-21T07:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>waiting_assignment</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>2026-09-21T09:00:00+03:00</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>2026-09-21T13:00:00+03:00</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
         <is>
           <t>45</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>1</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -3728,85 +3798,120 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>waiting_assignment</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>2026-09-21T10:00:00+03:00</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>2026-09-21T10:30:00+03:00</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
         <is>
           <t>60</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>1</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -3836,85 +3941,120 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-09-21T09:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>waiting_assignment</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>2026-09-21T11:00:00+03:00</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>2026-09-21T15:00:00+03:00</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
         <is>
           <t>90</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>1</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -3944,85 +4084,120 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-09-21T10:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>waiting_assignment</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>2026-09-21T12:00:00+03:00</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>2026-09-21T16:00:00+03:00</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>1</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
         <is>
           <t>4</t>
         </is>
@@ -4052,85 +4227,120 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-09-21T11:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>waiting_assignment</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>2026-09-21T13:00:00+03:00</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>2026-09-21T17:00:00+03:00</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
         <is>
           <t>45</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>1</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
         <is>
           <t>5</t>
         </is>
@@ -4160,85 +4370,120 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-09-21T12:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>waiting_assignment</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>2026-09-21T14:00:00+03:00</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>2026-09-21T18:00:00+03:00</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
         <is>
           <t>60</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>1</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -4268,85 +4513,120 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-09-21T13:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>waiting_assignment</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>2026-09-21T15:00:00+03:00</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>2026-09-21T19:00:00+03:00</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
         <is>
           <t>90</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>1</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -4376,85 +4656,120 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2026-09-21T20:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
           <t>in_progress</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>in_progress</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>2026-09-21T22:00:00+03:00</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t>2026-09-22T02:00:00+03:00</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="P9" t="inlineStr">
         <is>
           <t>2026-09-21T22:10:00+03:00</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="Q9" t="inlineStr">
         <is>
           <t>2026-09-21T22:40:00+03:00</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="R9" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
         <is>
           <t>2026-09-21T22:00:00+03:00</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="S9" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="T9" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr">
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
         <is>
           <t>8</t>
         </is>
@@ -4484,85 +4799,120 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2026-09-21T07:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
           <t>in_progress</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>in_progress</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>2026-09-21T09:00:00+03:00</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>2026-09-21T13:00:00+03:00</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="P10" t="inlineStr">
         <is>
           <t>2026-09-21T09:10:00+03:00</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="Q10" t="inlineStr">
         <is>
           <t>2026-09-21T09:55:00+03:00</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="R10" t="inlineStr">
         <is>
           <t>45</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
         <is>
           <t>2026-09-21T09:00:00+03:00</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="T10" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr">
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
         <is>
           <t>9</t>
         </is>
@@ -4592,85 +4942,120 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
           <t>in_progress</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>in_progress</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>2026-09-21T10:00:00+03:00</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>2026-09-21T10:30:00+03:00</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="P11" t="inlineStr">
         <is>
           <t>2026-09-21T10:10:00+03:00</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="Q11" t="inlineStr">
         <is>
           <t>2026-09-21T11:10:00+03:00</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="R11" t="inlineStr">
         <is>
           <t>60</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
         <is>
           <t>2026-09-21T10:00:00+03:00</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="T11" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="U11" t="inlineStr">
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr">
         <is>
           <t>10</t>
         </is>
@@ -4700,85 +5085,120 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2026-09-21T09:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
           <t>in_progress</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>in_progress</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>2026-09-21T11:00:00+03:00</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="O12" t="inlineStr">
         <is>
           <t>2026-09-21T15:00:00+03:00</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="P12" t="inlineStr">
         <is>
           <t>2026-09-21T11:10:00+03:00</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="Q12" t="inlineStr">
         <is>
           <t>2026-09-21T12:40:00+03:00</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="R12" t="inlineStr">
         <is>
           <t>90</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
         <is>
           <t>2026-09-21T11:00:00+03:00</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="R12" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="S12" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="T12" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="U12" t="inlineStr">
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AB12" t="inlineStr">
         <is>
           <t>11</t>
         </is>
@@ -4808,85 +5228,120 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2026-09-21T10:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
           <t>in_progress</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>in_progress</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>2026-09-21T12:00:00+03:00</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="O13" t="inlineStr">
         <is>
           <t>2026-09-21T16:00:00+03:00</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="P13" t="inlineStr">
         <is>
           <t>2026-09-21T12:10:00+03:00</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="Q13" t="inlineStr">
         <is>
           <t>2026-09-21T12:40:00+03:00</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="R13" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
         <is>
           <t>2026-09-21T12:00:00+03:00</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="S13" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="T13" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="U13" t="inlineStr">
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AB13" t="inlineStr">
         <is>
           <t>12</t>
         </is>
@@ -4916,85 +5371,120 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2026-09-21T11:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
           <t>in_progress</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="M14" t="inlineStr">
         <is>
           <t>in_progress</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="N14" t="inlineStr">
         <is>
           <t>2026-09-21T13:00:00+03:00</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="O14" t="inlineStr">
         <is>
           <t>2026-09-21T17:00:00+03:00</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="P14" t="inlineStr">
         <is>
           <t>2026-09-21T13:10:00+03:00</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="Q14" t="inlineStr">
         <is>
           <t>2026-09-21T13:55:00+03:00</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="R14" t="inlineStr">
         <is>
           <t>45</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr">
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
         <is>
           <t>2026-09-21T13:00:00+03:00</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="S14" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="T14" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="U14" t="inlineStr">
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AB14" t="inlineStr">
         <is>
           <t>13</t>
         </is>
@@ -5024,85 +5514,120 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2026-09-21T12:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
           <t>in_progress</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>in_progress</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t>2026-09-21T14:00:00+03:00</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="O15" t="inlineStr">
         <is>
           <t>2026-09-21T18:00:00+03:00</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="P15" t="inlineStr">
         <is>
           <t>2026-09-21T14:10:00+03:00</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="Q15" t="inlineStr">
         <is>
           <t>2026-09-21T15:10:00+03:00</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="R15" t="inlineStr">
         <is>
           <t>60</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
         <is>
           <t>2026-09-21T14:00:00+03:00</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="S15" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="T15" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="U15" t="inlineStr">
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AB15" t="inlineStr">
         <is>
           <t>14</t>
         </is>
@@ -5132,85 +5657,120 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2026-09-21T13:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
           <t>in_progress</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="M16" t="inlineStr">
         <is>
           <t>in_progress</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="N16" t="inlineStr">
         <is>
           <t>2026-09-21T15:00:00+03:00</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="O16" t="inlineStr">
         <is>
           <t>2026-09-21T19:00:00+03:00</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="P16" t="inlineStr">
         <is>
           <t>2026-09-21T15:10:00+03:00</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="Q16" t="inlineStr">
         <is>
           <t>2026-09-21T16:40:00+03:00</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="R16" t="inlineStr">
         <is>
           <t>90</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="O16" t="inlineStr">
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
         <is>
           <t>2026-09-21T15:00:00+03:00</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="S16" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="T16" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="U16" t="inlineStr">
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AB16" t="inlineStr">
         <is>
           <t>15</t>
         </is>
@@ -5240,85 +5800,120 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2026-09-21T20:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="M17" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="N17" t="inlineStr">
         <is>
           <t>2026-09-21T22:00:00+03:00</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="O17" t="inlineStr">
         <is>
           <t>2026-09-22T02:00:00+03:00</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="P17" t="inlineStr">
         <is>
           <t>2026-09-21T22:10:00+03:00</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="Q17" t="inlineStr">
         <is>
           <t>2026-09-21T22:40:00+03:00</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="R17" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
+      <c r="S17" t="inlineStr">
         <is>
           <t>46</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr">
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
         <is>
           <t>2026-09-21T22:00:00+03:00</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr">
+      <c r="W17" t="inlineStr">
         <is>
           <t>2026-09-21T22:30:00+03:00</t>
         </is>
       </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="S17" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="T17" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="U17" t="inlineStr">
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AB17" t="inlineStr">
         <is>
           <t>16</t>
         </is>
@@ -5348,85 +5943,120 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2026-09-21T07:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="M18" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="N18" t="inlineStr">
         <is>
           <t>2026-09-21T09:00:00+03:00</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="O18" t="inlineStr">
         <is>
           <t>2026-09-21T13:00:00+03:00</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="P18" t="inlineStr">
         <is>
           <t>2026-09-21T09:10:00+03:00</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="Q18" t="inlineStr">
         <is>
           <t>2026-09-21T09:55:00+03:00</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="R18" t="inlineStr">
         <is>
           <t>45</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="S18" t="inlineStr">
         <is>
           <t>62</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="O18" t="inlineStr">
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
         <is>
           <t>2026-09-21T09:00:00+03:00</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr">
+      <c r="W18" t="inlineStr">
         <is>
           <t>2026-09-21T09:45:00+03:00</t>
         </is>
       </c>
-      <c r="Q18" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="R18" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="S18" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="T18" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="U18" t="inlineStr">
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AB18" t="inlineStr">
         <is>
           <t>17</t>
         </is>
@@ -5456,85 +6086,120 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="M19" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="N19" t="inlineStr">
         <is>
           <t>2026-09-21T10:00:00+03:00</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="O19" t="inlineStr">
         <is>
           <t>2026-09-21T10:30:00+03:00</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="P19" t="inlineStr">
         <is>
           <t>2026-09-21T10:10:00+03:00</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="Q19" t="inlineStr">
         <is>
           <t>2026-09-21T11:10:00+03:00</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="R19" t="inlineStr">
         <is>
           <t>60</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
+      <c r="S19" t="inlineStr">
         <is>
           <t>78</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="O19" t="inlineStr">
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
         <is>
           <t>2026-09-21T10:00:00+03:00</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr">
+      <c r="W19" t="inlineStr">
         <is>
           <t>2026-09-21T11:00:00+03:00</t>
         </is>
       </c>
-      <c r="Q19" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="R19" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="S19" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="T19" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="U19" t="inlineStr">
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AB19" t="inlineStr">
         <is>
           <t>18</t>
         </is>
@@ -5564,85 +6229,120 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>2026-09-21T09:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="M20" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="N20" t="inlineStr">
         <is>
           <t>2026-09-21T11:00:00+03:00</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="O20" t="inlineStr">
         <is>
           <t>2026-09-21T15:00:00+03:00</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="P20" t="inlineStr">
         <is>
           <t>2026-09-21T11:10:00+03:00</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="Q20" t="inlineStr">
         <is>
           <t>2026-09-21T12:40:00+03:00</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
+      <c r="R20" t="inlineStr">
         <is>
           <t>90</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr">
+      <c r="S20" t="inlineStr">
         <is>
           <t>109</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="O20" t="inlineStr">
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
         <is>
           <t>2026-09-21T11:00:00+03:00</t>
         </is>
       </c>
-      <c r="P20" t="inlineStr">
+      <c r="W20" t="inlineStr">
         <is>
           <t>2026-09-21T12:30:00+03:00</t>
         </is>
       </c>
-      <c r="Q20" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="R20" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="S20" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="T20" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="U20" t="inlineStr">
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AB20" t="inlineStr">
         <is>
           <t>19</t>
         </is>
@@ -5672,85 +6372,120 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>2026-09-21T10:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="M21" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="N21" t="inlineStr">
         <is>
           <t>2026-09-21T12:00:00+03:00</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="O21" t="inlineStr">
         <is>
           <t>2026-09-21T16:00:00+03:00</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="P21" t="inlineStr">
         <is>
           <t>2026-09-21T12:10:00+03:00</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="Q21" t="inlineStr">
         <is>
           <t>2026-09-21T12:40:00+03:00</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="R21" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr">
+      <c r="S21" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="O21" t="inlineStr">
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
         <is>
           <t>2026-09-21T12:00:00+03:00</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr">
+      <c r="W21" t="inlineStr">
         <is>
           <t>2026-09-21T12:30:00+03:00</t>
         </is>
       </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="S21" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="T21" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="U21" t="inlineStr">
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AA21" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AB21" t="inlineStr">
         <is>
           <t>20</t>
         </is>
@@ -5780,85 +6515,120 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>2026-09-21T11:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="M22" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="N22" t="inlineStr">
         <is>
           <t>2026-09-21T13:00:00+03:00</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="O22" t="inlineStr">
         <is>
           <t>2026-09-21T17:00:00+03:00</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="P22" t="inlineStr">
         <is>
           <t>2026-09-21T13:10:00+03:00</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="Q22" t="inlineStr">
         <is>
           <t>2026-09-21T13:55:00+03:00</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr">
+      <c r="R22" t="inlineStr">
         <is>
           <t>45</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr">
+      <c r="S22" t="inlineStr">
         <is>
           <t>46</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="O22" t="inlineStr">
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
         <is>
           <t>2026-09-21T13:00:00+03:00</t>
         </is>
       </c>
-      <c r="P22" t="inlineStr">
+      <c r="W22" t="inlineStr">
         <is>
           <t>2026-09-21T13:45:00+03:00</t>
         </is>
       </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="S22" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="T22" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="U22" t="inlineStr">
+      <c r="X22" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Z22" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AB22" t="inlineStr">
         <is>
           <t>21</t>
         </is>
@@ -5888,85 +6658,120 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>2026-09-21T12:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="M23" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="N23" t="inlineStr">
         <is>
           <t>2026-09-21T14:00:00+03:00</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="O23" t="inlineStr">
         <is>
           <t>2026-09-21T18:00:00+03:00</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="P23" t="inlineStr">
         <is>
           <t>2026-09-21T14:10:00+03:00</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="Q23" t="inlineStr">
         <is>
           <t>2026-09-21T15:10:00+03:00</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
+      <c r="R23" t="inlineStr">
         <is>
           <t>60</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr">
+      <c r="S23" t="inlineStr">
         <is>
           <t>62</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="O23" t="inlineStr">
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
         <is>
           <t>2026-09-21T14:00:00+03:00</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr">
+      <c r="W23" t="inlineStr">
         <is>
           <t>2026-09-21T15:00:00+03:00</t>
         </is>
       </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="R23" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="S23" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="T23" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="U23" t="inlineStr">
+      <c r="X23" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Z23" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AB23" t="inlineStr">
         <is>
           <t>22</t>
         </is>
@@ -5996,85 +6801,120 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>2026-09-21T13:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="M24" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="N24" t="inlineStr">
         <is>
           <t>2026-09-21T15:00:00+03:00</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="O24" t="inlineStr">
         <is>
           <t>2026-09-21T19:00:00+03:00</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
+      <c r="P24" t="inlineStr">
         <is>
           <t>2026-09-21T15:10:00+03:00</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="Q24" t="inlineStr">
         <is>
           <t>2026-09-21T16:40:00+03:00</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
+      <c r="R24" t="inlineStr">
         <is>
           <t>90</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr">
+      <c r="S24" t="inlineStr">
         <is>
           <t>93</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="O24" t="inlineStr">
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
         <is>
           <t>2026-09-21T15:00:00+03:00</t>
         </is>
       </c>
-      <c r="P24" t="inlineStr">
+      <c r="W24" t="inlineStr">
         <is>
           <t>2026-09-21T16:30:00+03:00</t>
         </is>
       </c>
-      <c r="Q24" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="R24" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="S24" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="T24" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="U24" t="inlineStr">
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Z24" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AB24" t="inlineStr">
         <is>
           <t>23</t>
         </is>
@@ -6104,85 +6944,120 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>2026-09-21T20:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
           <t>wont_fix</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="M25" t="inlineStr">
         <is>
           <t>cancelled</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="N25" t="inlineStr">
         <is>
           <t>2026-09-21T22:00:00+03:00</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="O25" t="inlineStr">
         <is>
           <t>2026-09-22T02:00:00+03:00</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="Q25" t="inlineStr">
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="X25" t="inlineStr">
         <is>
           <t>Синтетическая отмена</t>
         </is>
       </c>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="S25" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="T25" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="U25" t="inlineStr">
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Z25" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AB25" t="inlineStr">
         <is>
           <t>24</t>
         </is>
@@ -13593,7 +14468,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>{"type":"FeatureCollection","properties":{"worker_id":9,"route_date":"2026-09-21","route_number":1},"features":[{"type":"Feature","geometry":{"type":"Point","coordinates":[37.748283,55.650237]},"properties":{"location_id":1,"ticket_id":null,"arrival_at":"2026-09-21T22:41:00+03:00","sequence":1}},{"type":"Feature","geometry":{"type":"Point","coordinates":[37.472323,55.806319]},"properties":{"location_id":2,"ticket_id":null,"arrival_at":"2026-09-21T23:21:00+03:00","sequence":2}},{"type":"Feature","geometry":{"type":"LineString","coordinates":[[37.748283,55.650237],[37.472323,55.806319]]},"properties":{"kind":"path","source":"straight_lines"}}]}</t>
+          <t>{"type":"FeatureCollection","properties":{"worker_id":9,"route_date":"2026-09-21","route_number":1},"features":[{"type":"Feature","geometry":{"type":"Point","coordinates":[37.748283,55.650237]},"properties":{"location_id":1,"ticket_id":null,"arrival_at":"2026-09-21T22:41:00+03:00","sequence":1,"service_start_at":"2026-09-21T22:41:00+03:00","service_end_at":"2026-09-21T23:11:00+03:00","waiting_minutes":0,"effective_service_minutes":null,"duration_source":"ticket_estimate"}},{"type":"Feature","geometry":{"type":"Point","coordinates":[37.472323,55.806319]},"properties":{"location_id":2,"ticket_id":null,"arrival_at":"2026-09-21T23:21:00+03:00","sequence":2,"service_start_at":"2026-09-21T23:21:00+03:00","service_end_at":"2026-09-21T23:51:00+03:00","waiting_minutes":0,"effective_service_minutes":null,"duration_source":"ticket_estimate"}},{"type":"Feature","geometry":{"type":"LineString","coordinates":[[37.748283,55.650237],[37.472323,55.806319]]},"properties":{"kind":"path","source":"straight_lines"}}]}</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -13625,7 +14500,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>{"type":"FeatureCollection","properties":{"worker_id":9,"route_date":"2026-09-21","route_number":2},"features":[{"type":"Feature","geometry":{"type":"Point","coordinates":[37.748283,55.650237]},"properties":{"location_id":1,"ticket_id":null,"arrival_at":"2026-09-21T22:42:00+03:00","sequence":1}},{"type":"Feature","geometry":{"type":"Point","coordinates":[37.472323,55.806319]},"properties":{"location_id":2,"ticket_id":null,"arrival_at":"2026-09-21T23:22:00+03:00","sequence":2}},{"type":"Feature","geometry":{"type":"LineString","coordinates":[[37.748283,55.650237],[37.472323,55.806319]]},"properties":{"kind":"path","source":"straight_lines"}}]}</t>
+          <t>{"type":"FeatureCollection","properties":{"worker_id":9,"route_date":"2026-09-21","route_number":2},"features":[{"type":"Feature","geometry":{"type":"Point","coordinates":[37.748283,55.650237]},"properties":{"location_id":1,"ticket_id":null,"arrival_at":"2026-09-21T22:42:00+03:00","sequence":1,"service_start_at":"2026-09-21T22:42:00+03:00","service_end_at":"2026-09-21T23:12:00+03:00","waiting_minutes":0,"effective_service_minutes":null,"duration_source":"ticket_estimate"}},{"type":"Feature","geometry":{"type":"Point","coordinates":[37.472323,55.806319]},"properties":{"location_id":2,"ticket_id":null,"arrival_at":"2026-09-21T23:22:00+03:00","sequence":2,"service_start_at":"2026-09-21T23:22:00+03:00","service_end_at":"2026-09-21T23:52:00+03:00","waiting_minutes":0,"effective_service_minutes":null,"duration_source":"ticket_estimate"}},{"type":"Feature","geometry":{"type":"LineString","coordinates":[[37.748283,55.650237],[37.472323,55.806319]]},"properties":{"kind":"path","source":"straight_lines"}}]}</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -13657,7 +14532,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>{"type":"FeatureCollection","properties":{"worker_id":10,"route_date":"2026-09-21","route_number":1},"features":[{"type":"Feature","geometry":{"type":"Point","coordinates":[37.472323,55.806319]},"properties":{"location_id":2,"ticket_id":null,"arrival_at":"2026-09-21T09:41:00+03:00","sequence":1}},{"type":"Feature","geometry":{"type":"Point","coordinates":[37.534812,55.791722]},"properties":{"location_id":3,"ticket_id":null,"arrival_at":"2026-09-21T10:21:00+03:00","sequence":2}},{"type":"Feature","geometry":{"type":"LineString","coordinates":[[37.472323,55.806319],[37.534812,55.791722]]},"properties":{"kind":"path","source":"straight_lines"}}]}</t>
+          <t>{"type":"FeatureCollection","properties":{"worker_id":10,"route_date":"2026-09-21","route_number":1},"features":[{"type":"Feature","geometry":{"type":"Point","coordinates":[37.472323,55.806319]},"properties":{"location_id":2,"ticket_id":null,"arrival_at":"2026-09-21T09:41:00+03:00","sequence":1,"service_start_at":"2026-09-21T09:41:00+03:00","service_end_at":"2026-09-21T10:11:00+03:00","waiting_minutes":0,"effective_service_minutes":null,"duration_source":"ticket_estimate"}},{"type":"Feature","geometry":{"type":"Point","coordinates":[37.534812,55.791722]},"properties":{"location_id":3,"ticket_id":null,"arrival_at":"2026-09-21T10:21:00+03:00","sequence":2,"service_start_at":"2026-09-21T10:21:00+03:00","service_end_at":"2026-09-21T10:51:00+03:00","waiting_minutes":0,"effective_service_minutes":null,"duration_source":"ticket_estimate"}},{"type":"Feature","geometry":{"type":"LineString","coordinates":[[37.472323,55.806319],[37.534812,55.791722]]},"properties":{"kind":"path","source":"straight_lines"}}]}</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -13689,7 +14564,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>{"type":"FeatureCollection","properties":{"worker_id":10,"route_date":"2026-09-21","route_number":2},"features":[{"type":"Feature","geometry":{"type":"Point","coordinates":[37.472323,55.806319]},"properties":{"location_id":2,"ticket_id":null,"arrival_at":"2026-09-21T09:42:00+03:00","sequence":1}},{"type":"Feature","geometry":{"type":"Point","coordinates":[37.534812,55.791722]},"properties":{"location_id":3,"ticket_id":null,"arrival_at":"2026-09-21T10:22:00+03:00","sequence":2}},{"type":"Feature","geometry":{"type":"LineString","coordinates":[[37.472323,55.806319],[37.534812,55.791722]]},"properties":{"kind":"path","source":"straight_lines"}}]}</t>
+          <t>{"type":"FeatureCollection","properties":{"worker_id":10,"route_date":"2026-09-21","route_number":2},"features":[{"type":"Feature","geometry":{"type":"Point","coordinates":[37.472323,55.806319]},"properties":{"location_id":2,"ticket_id":null,"arrival_at":"2026-09-21T09:42:00+03:00","sequence":1,"service_start_at":"2026-09-21T09:42:00+03:00","service_end_at":"2026-09-21T10:12:00+03:00","waiting_minutes":0,"effective_service_minutes":null,"duration_source":"ticket_estimate"}},{"type":"Feature","geometry":{"type":"Point","coordinates":[37.534812,55.791722]},"properties":{"location_id":3,"ticket_id":null,"arrival_at":"2026-09-21T10:22:00+03:00","sequence":2,"service_start_at":"2026-09-21T10:22:00+03:00","service_end_at":"2026-09-21T10:52:00+03:00","waiting_minutes":0,"effective_service_minutes":null,"duration_source":"ticket_estimate"}},{"type":"Feature","geometry":{"type":"LineString","coordinates":[[37.472323,55.806319],[37.534812,55.791722]]},"properties":{"kind":"path","source":"straight_lines"}}]}</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -13721,7 +14596,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>{"type":"FeatureCollection","properties":{"worker_id":11,"route_date":"2026-09-21","route_number":1},"features":[{"type":"Feature","geometry":{"type":"Point","coordinates":[37.534812,55.791722]},"properties":{"location_id":3,"ticket_id":null,"arrival_at":"2026-09-21T09:41:00+03:00","sequence":1}},{"type":"Feature","geometry":{"type":"Point","coordinates":[37.552259,55.717344]},"properties":{"location_id":4,"ticket_id":null,"arrival_at":"2026-09-21T10:21:00+03:00","sequence":2}},{"type":"Feature","geometry":{"type":"LineString","coordinates":[[37.534812,55.791722],[37.552259,55.717344]]},"properties":{"kind":"path","source":"straight_lines"}}]}</t>
+          <t>{"type":"FeatureCollection","properties":{"worker_id":11,"route_date":"2026-09-21","route_number":1},"features":[{"type":"Feature","geometry":{"type":"Point","coordinates":[37.534812,55.791722]},"properties":{"location_id":3,"ticket_id":null,"arrival_at":"2026-09-21T09:41:00+03:00","sequence":1,"service_start_at":"2026-09-21T09:41:00+03:00","service_end_at":"2026-09-21T10:11:00+03:00","waiting_minutes":0,"effective_service_minutes":null,"duration_source":"ticket_estimate"}},{"type":"Feature","geometry":{"type":"Point","coordinates":[37.552259,55.717344]},"properties":{"location_id":4,"ticket_id":null,"arrival_at":"2026-09-21T10:21:00+03:00","sequence":2,"service_start_at":"2026-09-21T10:21:00+03:00","service_end_at":"2026-09-21T10:51:00+03:00","waiting_minutes":0,"effective_service_minutes":null,"duration_source":"ticket_estimate"}},{"type":"Feature","geometry":{"type":"LineString","coordinates":[[37.534812,55.791722],[37.552259,55.717344]]},"properties":{"kind":"path","source":"straight_lines"}}]}</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -13753,7 +14628,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>{"type":"FeatureCollection","properties":{"worker_id":11,"route_date":"2026-09-21","route_number":2},"features":[{"type":"Feature","geometry":{"type":"Point","coordinates":[37.534812,55.791722]},"properties":{"location_id":3,"ticket_id":null,"arrival_at":"2026-09-21T09:42:00+03:00","sequence":1}},{"type":"Feature","geometry":{"type":"Point","coordinates":[37.552259,55.717344]},"properties":{"location_id":4,"ticket_id":null,"arrival_at":"2026-09-21T10:22:00+03:00","sequence":2}},{"type":"Feature","geometry":{"type":"LineString","coordinates":[[37.534812,55.791722],[37.552259,55.717344]]},"properties":{"kind":"path","source":"straight_lines"}}]}</t>
+          <t>{"type":"FeatureCollection","properties":{"worker_id":11,"route_date":"2026-09-21","route_number":2},"features":[{"type":"Feature","geometry":{"type":"Point","coordinates":[37.534812,55.791722]},"properties":{"location_id":3,"ticket_id":null,"arrival_at":"2026-09-21T09:42:00+03:00","sequence":1,"service_start_at":"2026-09-21T09:42:00+03:00","service_end_at":"2026-09-21T10:12:00+03:00","waiting_minutes":0,"effective_service_minutes":null,"duration_source":"ticket_estimate"}},{"type":"Feature","geometry":{"type":"Point","coordinates":[37.552259,55.717344]},"properties":{"location_id":4,"ticket_id":null,"arrival_at":"2026-09-21T10:22:00+03:00","sequence":2,"service_start_at":"2026-09-21T10:22:00+03:00","service_end_at":"2026-09-21T10:52:00+03:00","waiting_minutes":0,"effective_service_minutes":null,"duration_source":"ticket_estimate"}},{"type":"Feature","geometry":{"type":"LineString","coordinates":[[37.534812,55.791722],[37.552259,55.717344]]},"properties":{"kind":"path","source":"straight_lines"}}]}</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -13785,7 +14660,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>{"type":"FeatureCollection","properties":{"worker_id":12,"route_date":"2026-09-21","route_number":1},"features":[{"type":"Feature","geometry":{"type":"Point","coordinates":[37.552259,55.717344]},"properties":{"location_id":4,"ticket_id":null,"arrival_at":"2026-09-21T09:41:00+03:00","sequence":1}},{"type":"Feature","geometry":{"type":"Point","coordinates":[37.496224,55.755907]},"properties":{"location_id":5,"ticket_id":null,"arrival_at":"2026-09-21T10:21:00+03:00","sequence":2}},{"type":"Feature","geometry":{"type":"LineString","coordinates":[[37.552259,55.717344],[37.496224,55.755907]]},"properties":{"kind":"path","source":"straight_lines"}}]}</t>
+          <t>{"type":"FeatureCollection","properties":{"worker_id":12,"route_date":"2026-09-21","route_number":1},"features":[{"type":"Feature","geometry":{"type":"Point","coordinates":[37.552259,55.717344]},"properties":{"location_id":4,"ticket_id":null,"arrival_at":"2026-09-21T09:41:00+03:00","sequence":1,"service_start_at":"2026-09-21T09:41:00+03:00","service_end_at":"2026-09-21T10:11:00+03:00","waiting_minutes":0,"effective_service_minutes":null,"duration_source":"ticket_estimate"}},{"type":"Feature","geometry":{"type":"Point","coordinates":[37.496224,55.755907]},"properties":{"location_id":5,"ticket_id":null,"arrival_at":"2026-09-21T10:21:00+03:00","sequence":2,"service_start_at":"2026-09-21T10:21:00+03:00","service_end_at":"2026-09-21T10:51:00+03:00","waiting_minutes":0,"effective_service_minutes":null,"duration_source":"ticket_estimate"}},{"type":"Feature","geometry":{"type":"LineString","coordinates":[[37.552259,55.717344],[37.496224,55.755907]]},"properties":{"kind":"path","source":"straight_lines"}}]}</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -13817,7 +14692,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>{"type":"FeatureCollection","properties":{"worker_id":12,"route_date":"2026-09-21","route_number":2},"features":[{"type":"Feature","geometry":{"type":"Point","coordinates":[37.552259,55.717344]},"properties":{"location_id":4,"ticket_id":null,"arrival_at":"2026-09-21T09:42:00+03:00","sequence":1}},{"type":"Feature","geometry":{"type":"Point","coordinates":[37.496224,55.755907]},"properties":{"location_id":5,"ticket_id":null,"arrival_at":"2026-09-21T10:22:00+03:00","sequence":2}},{"type":"Feature","geometry":{"type":"LineString","coordinates":[[37.552259,55.717344],[37.496224,55.755907]]},"properties":{"kind":"path","source":"straight_lines"}}]}</t>
+          <t>{"type":"FeatureCollection","properties":{"worker_id":12,"route_date":"2026-09-21","route_number":2},"features":[{"type":"Feature","geometry":{"type":"Point","coordinates":[37.552259,55.717344]},"properties":{"location_id":4,"ticket_id":null,"arrival_at":"2026-09-21T09:42:00+03:00","sequence":1,"service_start_at":"2026-09-21T09:42:00+03:00","service_end_at":"2026-09-21T10:12:00+03:00","waiting_minutes":0,"effective_service_minutes":null,"duration_source":"ticket_estimate"}},{"type":"Feature","geometry":{"type":"Point","coordinates":[37.496224,55.755907]},"properties":{"location_id":5,"ticket_id":null,"arrival_at":"2026-09-21T10:22:00+03:00","sequence":2,"service_start_at":"2026-09-21T10:22:00+03:00","service_end_at":"2026-09-21T10:52:00+03:00","waiting_minutes":0,"effective_service_minutes":null,"duration_source":"ticket_estimate"}},{"type":"Feature","geometry":{"type":"LineString","coordinates":[[37.552259,55.717344],[37.496224,55.755907]]},"properties":{"kind":"path","source":"straight_lines"}}]}</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -14411,25 +15286,40 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>default_priority</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>travel_minutes</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>work_minutes</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>documents_minutes</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>norm_minutes</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
@@ -14443,25 +15333,40 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>synthetic_906_1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>15</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>55</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -14475,25 +15380,40 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>synthetic_906_2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
           <t>15</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>55</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -14507,25 +15427,40 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>synthetic_906_3</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
           <t>15</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>55</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>3</t>
         </is>

</xml_diff>

<commit_message>
Regenerate synthetic data without ticket_assignments (T07)
</commit_message>
<xml_diff>
--- a/backend/bruno/fixtures/dataset.xlsx
+++ b/backend/bruno/fixtures/dataset.xlsx
@@ -30,14 +30,13 @@
     <sheet name="brigades" sheetId="21" state="visible" r:id="rId21"/>
     <sheet name="notification_events" sheetId="22" state="visible" r:id="rId22"/>
     <sheet name="ticket_appliances" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="ticket_assignments" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="ticket_comments" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="work_events" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="worker_day_states" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="brigade_members" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="day_plan_revisions" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="equipment_movements" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet name="routes" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="ticket_comments" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="work_events" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="worker_day_states" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="brigade_members" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="day_plan_revisions" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="equipment_movements" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="routes" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3557,75 +3556,85 @@
       </c>
       <c r="N1" t="inlineStr">
         <is>
+          <t>assigned_worker_id</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>is_pinned</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
           <t>visit_window_start</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>visit_window_end</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>planned_start_at</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>planned_end_at</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>estimated_duration_minutes</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>actual_duration_minutes</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>revision</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>execution_cycle</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>actual_started_at</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>actual_completed_at</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>cancel_reason</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>last_event_id</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>created_at</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>updated_at</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
@@ -3700,52 +3709,52 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
           <t>2026-09-21T09:00:00+03:00</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>2026-09-21T13:00:00+03:00</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
       <c r="R2" t="inlineStr">
         <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
           <t>45</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>\N</t>
+          <t>1</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>\N</t>
+          <t>1</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
@@ -3760,15 +3769,25 @@
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -3843,52 +3862,52 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
           <t>2026-09-21T10:00:00+03:00</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>2026-09-21T10:30:00+03:00</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
       <c r="R3" t="inlineStr">
         <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
           <t>60</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>\N</t>
+          <t>1</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>\N</t>
+          <t>1</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
@@ -3903,15 +3922,25 @@
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AB3" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -3986,52 +4015,52 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
           <t>2026-09-21T11:00:00+03:00</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>2026-09-21T15:00:00+03:00</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
       <c r="R4" t="inlineStr">
         <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
           <t>90</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>\N</t>
+          <t>1</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>\N</t>
+          <t>1</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
@@ -4046,15 +4075,25 @@
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AB4" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -4129,52 +4168,52 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
           <t>2026-09-21T12:00:00+03:00</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>2026-09-21T16:00:00+03:00</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
       <c r="R5" t="inlineStr">
         <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
           <t>30</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>\N</t>
+          <t>1</t>
         </is>
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>\N</t>
+          <t>1</t>
         </is>
       </c>
       <c r="X5" t="inlineStr">
@@ -4189,15 +4228,25 @@
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
         <is>
           <t>4</t>
         </is>
@@ -4272,52 +4321,52 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
           <t>2026-09-21T13:00:00+03:00</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>2026-09-21T17:00:00+03:00</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
       <c r="R6" t="inlineStr">
         <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
           <t>45</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>\N</t>
+          <t>1</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>\N</t>
+          <t>1</t>
         </is>
       </c>
       <c r="X6" t="inlineStr">
@@ -4332,15 +4381,25 @@
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AA6" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AB6" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
         <is>
           <t>5</t>
         </is>
@@ -4415,52 +4474,52 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
           <t>2026-09-21T14:00:00+03:00</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="Q7" t="inlineStr">
         <is>
           <t>2026-09-21T18:00:00+03:00</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
       <c r="R7" t="inlineStr">
         <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
           <t>60</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>\N</t>
+          <t>1</t>
         </is>
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>\N</t>
+          <t>1</t>
         </is>
       </c>
       <c r="X7" t="inlineStr">
@@ -4475,15 +4534,25 @@
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AA7" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AB7" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -4558,52 +4627,52 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
           <t>2026-09-21T15:00:00+03:00</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="Q8" t="inlineStr">
         <is>
           <t>2026-09-21T19:00:00+03:00</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
       <c r="R8" t="inlineStr">
         <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
           <t>90</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="T8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>\N</t>
+          <t>1</t>
         </is>
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>\N</t>
+          <t>1</t>
         </is>
       </c>
       <c r="X8" t="inlineStr">
@@ -4618,15 +4687,25 @@
       </c>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AA8" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AB8" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -4701,59 +4780,59 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
           <t>2026-09-21T22:00:00+03:00</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr">
+      <c r="Q9" t="inlineStr">
         <is>
           <t>2026-09-22T02:00:00+03:00</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr">
+      <c r="R9" t="inlineStr">
         <is>
           <t>2026-09-21T22:10:00+03:00</t>
         </is>
       </c>
-      <c r="Q9" t="inlineStr">
+      <c r="S9" t="inlineStr">
         <is>
           <t>2026-09-21T22:40:00+03:00</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr">
+      <c r="T9" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="S9" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="T9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
           <t>2026-09-21T22:00:00+03:00</t>
         </is>
       </c>
-      <c r="W9" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="X9" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
       <c r="Y9" t="inlineStr">
         <is>
           <t>\N</t>
@@ -4761,15 +4840,25 @@
       </c>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AA9" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AB9" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
         <is>
           <t>8</t>
         </is>
@@ -4844,59 +4933,59 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
           <t>2026-09-21T09:00:00+03:00</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr">
+      <c r="Q10" t="inlineStr">
         <is>
           <t>2026-09-21T13:00:00+03:00</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr">
+      <c r="R10" t="inlineStr">
         <is>
           <t>2026-09-21T09:10:00+03:00</t>
         </is>
       </c>
-      <c r="Q10" t="inlineStr">
+      <c r="S10" t="inlineStr">
         <is>
           <t>2026-09-21T09:55:00+03:00</t>
         </is>
       </c>
-      <c r="R10" t="inlineStr">
+      <c r="T10" t="inlineStr">
         <is>
           <t>45</t>
         </is>
       </c>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="T10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
           <t>2026-09-21T09:00:00+03:00</t>
         </is>
       </c>
-      <c r="W10" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="X10" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
       <c r="Y10" t="inlineStr">
         <is>
           <t>\N</t>
@@ -4904,15 +4993,25 @@
       </c>
       <c r="Z10" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AA10" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AB10" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
         <is>
           <t>9</t>
         </is>
@@ -4987,59 +5086,59 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
           <t>2026-09-21T10:00:00+03:00</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr">
+      <c r="Q11" t="inlineStr">
         <is>
           <t>2026-09-21T10:30:00+03:00</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr">
+      <c r="R11" t="inlineStr">
         <is>
           <t>2026-09-21T10:10:00+03:00</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr">
+      <c r="S11" t="inlineStr">
         <is>
           <t>2026-09-21T11:10:00+03:00</t>
         </is>
       </c>
-      <c r="R11" t="inlineStr">
+      <c r="T11" t="inlineStr">
         <is>
           <t>60</t>
         </is>
       </c>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="T11" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
           <t>2026-09-21T10:00:00+03:00</t>
         </is>
       </c>
-      <c r="W11" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="X11" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
       <c r="Y11" t="inlineStr">
         <is>
           <t>\N</t>
@@ -5047,15 +5146,25 @@
       </c>
       <c r="Z11" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AA11" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AB11" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
         <is>
           <t>10</t>
         </is>
@@ -5130,59 +5239,59 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
           <t>2026-09-21T11:00:00+03:00</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr">
+      <c r="Q12" t="inlineStr">
         <is>
           <t>2026-09-21T15:00:00+03:00</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr">
+      <c r="R12" t="inlineStr">
         <is>
           <t>2026-09-21T11:10:00+03:00</t>
         </is>
       </c>
-      <c r="Q12" t="inlineStr">
+      <c r="S12" t="inlineStr">
         <is>
           <t>2026-09-21T12:40:00+03:00</t>
         </is>
       </c>
-      <c r="R12" t="inlineStr">
+      <c r="T12" t="inlineStr">
         <is>
           <t>90</t>
         </is>
       </c>
-      <c r="S12" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="T12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
           <t>2026-09-21T11:00:00+03:00</t>
         </is>
       </c>
-      <c r="W12" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="X12" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
       <c r="Y12" t="inlineStr">
         <is>
           <t>\N</t>
@@ -5190,15 +5299,25 @@
       </c>
       <c r="Z12" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AA12" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AB12" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
         <is>
           <t>11</t>
         </is>
@@ -5273,59 +5392,59 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
           <t>2026-09-21T12:00:00+03:00</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr">
+      <c r="Q13" t="inlineStr">
         <is>
           <t>2026-09-21T16:00:00+03:00</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr">
+      <c r="R13" t="inlineStr">
         <is>
           <t>2026-09-21T12:10:00+03:00</t>
         </is>
       </c>
-      <c r="Q13" t="inlineStr">
+      <c r="S13" t="inlineStr">
         <is>
           <t>2026-09-21T12:40:00+03:00</t>
         </is>
       </c>
-      <c r="R13" t="inlineStr">
+      <c r="T13" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="S13" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="T13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
           <t>2026-09-21T12:00:00+03:00</t>
         </is>
       </c>
-      <c r="W13" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="X13" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
       <c r="Y13" t="inlineStr">
         <is>
           <t>\N</t>
@@ -5333,15 +5452,25 @@
       </c>
       <c r="Z13" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AA13" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AB13" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
         <is>
           <t>12</t>
         </is>
@@ -5416,59 +5545,59 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
           <t>2026-09-21T13:00:00+03:00</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr">
+      <c r="Q14" t="inlineStr">
         <is>
           <t>2026-09-21T17:00:00+03:00</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr">
+      <c r="R14" t="inlineStr">
         <is>
           <t>2026-09-21T13:10:00+03:00</t>
         </is>
       </c>
-      <c r="Q14" t="inlineStr">
+      <c r="S14" t="inlineStr">
         <is>
           <t>2026-09-21T13:55:00+03:00</t>
         </is>
       </c>
-      <c r="R14" t="inlineStr">
+      <c r="T14" t="inlineStr">
         <is>
           <t>45</t>
         </is>
       </c>
-      <c r="S14" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="T14" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
           <t>2026-09-21T13:00:00+03:00</t>
         </is>
       </c>
-      <c r="W14" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="X14" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
       <c r="Y14" t="inlineStr">
         <is>
           <t>\N</t>
@@ -5476,15 +5605,25 @@
       </c>
       <c r="Z14" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AA14" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AB14" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
         <is>
           <t>13</t>
         </is>
@@ -5559,59 +5698,59 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
           <t>2026-09-21T14:00:00+03:00</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr">
+      <c r="Q15" t="inlineStr">
         <is>
           <t>2026-09-21T18:00:00+03:00</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr">
+      <c r="R15" t="inlineStr">
         <is>
           <t>2026-09-21T14:10:00+03:00</t>
         </is>
       </c>
-      <c r="Q15" t="inlineStr">
+      <c r="S15" t="inlineStr">
         <is>
           <t>2026-09-21T15:10:00+03:00</t>
         </is>
       </c>
-      <c r="R15" t="inlineStr">
+      <c r="T15" t="inlineStr">
         <is>
           <t>60</t>
         </is>
       </c>
-      <c r="S15" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="T15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
           <t>2026-09-21T14:00:00+03:00</t>
         </is>
       </c>
-      <c r="W15" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="X15" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
       <c r="Y15" t="inlineStr">
         <is>
           <t>\N</t>
@@ -5619,15 +5758,25 @@
       </c>
       <c r="Z15" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AA15" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AB15" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AD15" t="inlineStr">
         <is>
           <t>14</t>
         </is>
@@ -5702,59 +5851,59 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
           <t>2026-09-21T15:00:00+03:00</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr">
+      <c r="Q16" t="inlineStr">
         <is>
           <t>2026-09-21T19:00:00+03:00</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr">
+      <c r="R16" t="inlineStr">
         <is>
           <t>2026-09-21T15:10:00+03:00</t>
         </is>
       </c>
-      <c r="Q16" t="inlineStr">
+      <c r="S16" t="inlineStr">
         <is>
           <t>2026-09-21T16:40:00+03:00</t>
         </is>
       </c>
-      <c r="R16" t="inlineStr">
+      <c r="T16" t="inlineStr">
         <is>
           <t>90</t>
         </is>
       </c>
-      <c r="S16" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="T16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
           <t>2026-09-21T15:00:00+03:00</t>
         </is>
       </c>
-      <c r="W16" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="X16" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
       <c r="Y16" t="inlineStr">
         <is>
           <t>\N</t>
@@ -5762,15 +5911,25 @@
       </c>
       <c r="Z16" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AA16" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AB16" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AD16" t="inlineStr">
         <is>
           <t>15</t>
         </is>
@@ -5845,75 +6004,85 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
           <t>2026-09-21T22:00:00+03:00</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr">
+      <c r="Q17" t="inlineStr">
         <is>
           <t>2026-09-22T02:00:00+03:00</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr">
+      <c r="R17" t="inlineStr">
         <is>
           <t>2026-09-21T22:10:00+03:00</t>
         </is>
       </c>
-      <c r="Q17" t="inlineStr">
+      <c r="S17" t="inlineStr">
         <is>
           <t>2026-09-21T22:40:00+03:00</t>
         </is>
       </c>
-      <c r="R17" t="inlineStr">
+      <c r="T17" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="S17" t="inlineStr">
+      <c r="U17" t="inlineStr">
         <is>
           <t>46</t>
         </is>
       </c>
-      <c r="T17" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="U17" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="V17" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
           <t>2026-09-21T22:00:00+03:00</t>
         </is>
       </c>
-      <c r="W17" t="inlineStr">
+      <c r="Y17" t="inlineStr">
         <is>
           <t>2026-09-21T22:30:00+03:00</t>
         </is>
       </c>
-      <c r="X17" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="Y17" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
       <c r="Z17" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AA17" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AB17" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr">
         <is>
           <t>16</t>
         </is>
@@ -5988,75 +6157,85 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
           <t>2026-09-21T09:00:00+03:00</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr">
+      <c r="Q18" t="inlineStr">
         <is>
           <t>2026-09-21T13:00:00+03:00</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr">
+      <c r="R18" t="inlineStr">
         <is>
           <t>2026-09-21T09:10:00+03:00</t>
         </is>
       </c>
-      <c r="Q18" t="inlineStr">
+      <c r="S18" t="inlineStr">
         <is>
           <t>2026-09-21T09:55:00+03:00</t>
         </is>
       </c>
-      <c r="R18" t="inlineStr">
+      <c r="T18" t="inlineStr">
         <is>
           <t>45</t>
         </is>
       </c>
-      <c r="S18" t="inlineStr">
+      <c r="U18" t="inlineStr">
         <is>
           <t>62</t>
         </is>
       </c>
-      <c r="T18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="U18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="V18" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
           <t>2026-09-21T09:00:00+03:00</t>
         </is>
       </c>
-      <c r="W18" t="inlineStr">
+      <c r="Y18" t="inlineStr">
         <is>
           <t>2026-09-21T09:45:00+03:00</t>
         </is>
       </c>
-      <c r="X18" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="Y18" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
       <c r="Z18" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AA18" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AB18" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AC18" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AD18" t="inlineStr">
         <is>
           <t>17</t>
         </is>
@@ -6131,75 +6310,85 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
           <t>2026-09-21T10:00:00+03:00</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr">
+      <c r="Q19" t="inlineStr">
         <is>
           <t>2026-09-21T10:30:00+03:00</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr">
+      <c r="R19" t="inlineStr">
         <is>
           <t>2026-09-21T10:10:00+03:00</t>
         </is>
       </c>
-      <c r="Q19" t="inlineStr">
+      <c r="S19" t="inlineStr">
         <is>
           <t>2026-09-21T11:10:00+03:00</t>
         </is>
       </c>
-      <c r="R19" t="inlineStr">
+      <c r="T19" t="inlineStr">
         <is>
           <t>60</t>
         </is>
       </c>
-      <c r="S19" t="inlineStr">
+      <c r="U19" t="inlineStr">
         <is>
           <t>78</t>
         </is>
       </c>
-      <c r="T19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="U19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="V19" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
           <t>2026-09-21T10:00:00+03:00</t>
         </is>
       </c>
-      <c r="W19" t="inlineStr">
+      <c r="Y19" t="inlineStr">
         <is>
           <t>2026-09-21T11:00:00+03:00</t>
         </is>
       </c>
-      <c r="X19" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="Y19" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
       <c r="Z19" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AA19" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AB19" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AC19" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AD19" t="inlineStr">
         <is>
           <t>18</t>
         </is>
@@ -6274,75 +6463,85 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
           <t>2026-09-21T11:00:00+03:00</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr">
+      <c r="Q20" t="inlineStr">
         <is>
           <t>2026-09-21T15:00:00+03:00</t>
         </is>
       </c>
-      <c r="P20" t="inlineStr">
+      <c r="R20" t="inlineStr">
         <is>
           <t>2026-09-21T11:10:00+03:00</t>
         </is>
       </c>
-      <c r="Q20" t="inlineStr">
+      <c r="S20" t="inlineStr">
         <is>
           <t>2026-09-21T12:40:00+03:00</t>
         </is>
       </c>
-      <c r="R20" t="inlineStr">
+      <c r="T20" t="inlineStr">
         <is>
           <t>90</t>
         </is>
       </c>
-      <c r="S20" t="inlineStr">
+      <c r="U20" t="inlineStr">
         <is>
           <t>109</t>
         </is>
       </c>
-      <c r="T20" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="U20" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="V20" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
           <t>2026-09-21T11:00:00+03:00</t>
         </is>
       </c>
-      <c r="W20" t="inlineStr">
+      <c r="Y20" t="inlineStr">
         <is>
           <t>2026-09-21T12:30:00+03:00</t>
         </is>
       </c>
-      <c r="X20" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="Y20" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
       <c r="Z20" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AA20" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AB20" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AC20" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AD20" t="inlineStr">
         <is>
           <t>19</t>
         </is>
@@ -6417,75 +6616,85 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
           <t>2026-09-21T12:00:00+03:00</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr">
+      <c r="Q21" t="inlineStr">
         <is>
           <t>2026-09-21T16:00:00+03:00</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr">
+      <c r="R21" t="inlineStr">
         <is>
           <t>2026-09-21T12:10:00+03:00</t>
         </is>
       </c>
-      <c r="Q21" t="inlineStr">
+      <c r="S21" t="inlineStr">
         <is>
           <t>2026-09-21T12:40:00+03:00</t>
         </is>
       </c>
-      <c r="R21" t="inlineStr">
+      <c r="T21" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="S21" t="inlineStr">
+      <c r="U21" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="T21" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="U21" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="V21" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
           <t>2026-09-21T12:00:00+03:00</t>
         </is>
       </c>
-      <c r="W21" t="inlineStr">
+      <c r="Y21" t="inlineStr">
         <is>
           <t>2026-09-21T12:30:00+03:00</t>
         </is>
       </c>
-      <c r="X21" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="Y21" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
       <c r="Z21" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AA21" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AB21" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AC21" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AD21" t="inlineStr">
         <is>
           <t>20</t>
         </is>
@@ -6560,75 +6769,85 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
           <t>2026-09-21T13:00:00+03:00</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr">
+      <c r="Q22" t="inlineStr">
         <is>
           <t>2026-09-21T17:00:00+03:00</t>
         </is>
       </c>
-      <c r="P22" t="inlineStr">
+      <c r="R22" t="inlineStr">
         <is>
           <t>2026-09-21T13:10:00+03:00</t>
         </is>
       </c>
-      <c r="Q22" t="inlineStr">
+      <c r="S22" t="inlineStr">
         <is>
           <t>2026-09-21T13:55:00+03:00</t>
         </is>
       </c>
-      <c r="R22" t="inlineStr">
+      <c r="T22" t="inlineStr">
         <is>
           <t>45</t>
         </is>
       </c>
-      <c r="S22" t="inlineStr">
+      <c r="U22" t="inlineStr">
         <is>
           <t>46</t>
         </is>
       </c>
-      <c r="T22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="U22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="V22" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X22" t="inlineStr">
+        <is>
           <t>2026-09-21T13:00:00+03:00</t>
         </is>
       </c>
-      <c r="W22" t="inlineStr">
+      <c r="Y22" t="inlineStr">
         <is>
           <t>2026-09-21T13:45:00+03:00</t>
         </is>
       </c>
-      <c r="X22" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="Y22" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
       <c r="Z22" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AA22" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AB22" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AC22" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AD22" t="inlineStr">
         <is>
           <t>21</t>
         </is>
@@ -6703,75 +6922,85 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
           <t>2026-09-21T14:00:00+03:00</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr">
+      <c r="Q23" t="inlineStr">
         <is>
           <t>2026-09-21T18:00:00+03:00</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr">
+      <c r="R23" t="inlineStr">
         <is>
           <t>2026-09-21T14:10:00+03:00</t>
         </is>
       </c>
-      <c r="Q23" t="inlineStr">
+      <c r="S23" t="inlineStr">
         <is>
           <t>2026-09-21T15:10:00+03:00</t>
         </is>
       </c>
-      <c r="R23" t="inlineStr">
+      <c r="T23" t="inlineStr">
         <is>
           <t>60</t>
         </is>
       </c>
-      <c r="S23" t="inlineStr">
+      <c r="U23" t="inlineStr">
         <is>
           <t>62</t>
         </is>
       </c>
-      <c r="T23" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="U23" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="V23" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X23" t="inlineStr">
+        <is>
           <t>2026-09-21T14:00:00+03:00</t>
         </is>
       </c>
-      <c r="W23" t="inlineStr">
+      <c r="Y23" t="inlineStr">
         <is>
           <t>2026-09-21T15:00:00+03:00</t>
         </is>
       </c>
-      <c r="X23" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="Y23" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
       <c r="Z23" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AC23" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AD23" t="inlineStr">
         <is>
           <t>22</t>
         </is>
@@ -6846,75 +7075,85 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
           <t>2026-09-21T15:00:00+03:00</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr">
+      <c r="Q24" t="inlineStr">
         <is>
           <t>2026-09-21T19:00:00+03:00</t>
         </is>
       </c>
-      <c r="P24" t="inlineStr">
+      <c r="R24" t="inlineStr">
         <is>
           <t>2026-09-21T15:10:00+03:00</t>
         </is>
       </c>
-      <c r="Q24" t="inlineStr">
+      <c r="S24" t="inlineStr">
         <is>
           <t>2026-09-21T16:40:00+03:00</t>
         </is>
       </c>
-      <c r="R24" t="inlineStr">
+      <c r="T24" t="inlineStr">
         <is>
           <t>90</t>
         </is>
       </c>
-      <c r="S24" t="inlineStr">
+      <c r="U24" t="inlineStr">
         <is>
           <t>93</t>
         </is>
       </c>
-      <c r="T24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="V24" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X24" t="inlineStr">
+        <is>
           <t>2026-09-21T15:00:00+03:00</t>
         </is>
       </c>
-      <c r="W24" t="inlineStr">
+      <c r="Y24" t="inlineStr">
         <is>
           <t>2026-09-21T16:30:00+03:00</t>
         </is>
       </c>
-      <c r="X24" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="Y24" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
       <c r="Z24" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AA24" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AB24" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AC24" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AD24" t="inlineStr">
         <is>
           <t>23</t>
         </is>
@@ -6989,75 +7228,85 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
           <t>2026-09-21T22:00:00+03:00</t>
         </is>
       </c>
-      <c r="O25" t="inlineStr">
+      <c r="Q25" t="inlineStr">
         <is>
           <t>2026-09-22T02:00:00+03:00</t>
         </is>
       </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
       <c r="R25" t="inlineStr">
         <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
           <t>30</t>
         </is>
       </c>
-      <c r="S25" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="T25" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>\N</t>
+          <t>1</t>
         </is>
       </c>
       <c r="W25" t="inlineStr">
         <is>
-          <t>\N</t>
+          <t>1</t>
         </is>
       </c>
       <c r="X25" t="inlineStr">
         <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Z25" t="inlineStr">
+        <is>
           <t>Синтетическая отмена</t>
         </is>
       </c>
-      <c r="Y25" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="Z25" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
       <c r="AA25" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="AB25" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AC25" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="AD25" t="inlineStr">
         <is>
           <t>24</t>
         </is>
@@ -13049,318 +13298,291 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>worker_id</t>
+          <t>author_id</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>assigned_at</t>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>updated_at</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>id</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>Синтетический комментарий 3, проверка UTF-8 и переноса
+второй строки</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Синтетический комментарий 6, проверка UTF-8 и переноса
+второй строки</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>2</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>Синтетический комментарий 9, проверка UTF-8 и переноса
+второй строки</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>Синтетический комментарий 12, проверка UTF-8 и переноса
+второй строки</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>4</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>Синтетический комментарий 15, проверка UTF-8 и переноса
+второй строки</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>5</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>Синтетический комментарий 18, проверка UTF-8 и переноса
+второй строки</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>6</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>21</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>Синтетический комментарий 21, проверка UTF-8 и переноса
+второй строки</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>7</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>24</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>Синтетический комментарий 24, проверка UTF-8 и переноса
+второй строки</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>8</t>
         </is>
       </c>
     </row>
@@ -13380,30 +13602,80 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>event_type</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>ticket_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>author_id</t>
-        </is>
-      </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>worker_id</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>district_id</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>updated_at</t>
+          <t>route_date</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
+        <is>
+          <t>occurred_at</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>recorded_at</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>actor_id</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>previous_state</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>new_state</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>before_revision</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>after_revision</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>idempotency_key</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>payload</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
@@ -13412,7 +13684,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>new_ticket</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -13422,254 +13694,72 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Синтетический комментарий 3, проверка UTF-8 и переноса
-второй строки</t>
+          <t>9</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Синтетический комментарий 6, проверка UTF-8 и переноса
-второй строки</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Синтетический комментарий 9, проверка UTF-8 и переноса
-второй строки</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Синтетический комментарий 12, проверка UTF-8 и переноса
-второй строки</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Синтетический комментарий 15, проверка UTF-8 и переноса
-второй строки</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Синтетический комментарий 18, проверка UTF-8 и переноса
-второй строки</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Синтетический комментарий 21, проверка UTF-8 и переноса
-второй строки</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Синтетический комментарий 24, проверка UTF-8 и переноса
-второй строки</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>8</t>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>waiting_assignment</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>synthetic-906-ticket-1</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>{"ticket_id":1}</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -13689,77 +13779,77 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>event_type</t>
+          <t>worker_id</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>ticket_id</t>
+          <t>district_id</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>worker_id</t>
+          <t>route_date</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>district_id</t>
+          <t>revision</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>route_date</t>
+          <t>available</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>occurred_at</t>
+          <t>unavailable_at</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>recorded_at</t>
+          <t>unavailable_until</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>actor_id</t>
+          <t>last_location_id</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>current_ticket_id</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>current_destination_id</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>en_route_started_at</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>expected_available_at</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
           <t>reason</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>previous_state</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>new_state</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>before_revision</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>after_revision</t>
-        </is>
-      </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>idempotency_key</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>payload</t>
+          <t>updated_at</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
@@ -13771,7 +13861,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>new_ticket</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -13781,7 +13871,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -13791,17 +13881,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>true</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00+03:00</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -13821,7 +13911,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>waiting_assignment</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -13831,17 +13921,17 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>\N</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>synthetic-906-ticket-1</t>
+          <t>2026-09-21T08:00:00+03:00</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>{"ticket_id":1}</t>
+          <t>2026-09-21T08:00:00+03:00</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -13866,164 +13956,60 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>brigade_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>worker_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>district_id</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>route_date</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>revision</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>available</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>unavailable_at</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>unavailable_until</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>last_location_id</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>current_ticket_id</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>current_destination_id</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>en_route_started_at</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>expected_available_at</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>reason</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>created_at</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>updated_at</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>id</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>9</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>1</t>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>12</t>
         </is>
       </c>
     </row>
@@ -14043,12 +14029,62 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>brigade_id</t>
+          <t>district_id</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>worker_id</t>
+          <t>route_date</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>revision</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>previous_revision</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>event_id</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>actor_id</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>fingerprint</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>diff</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>result</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>is_current</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>id</t>
         </is>
       </c>
     </row>
@@ -14060,43 +14096,57 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>9</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>12</t>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>93804b6a82cb845e7bf368040bd158224af7bfadb3a11d0a585f119745a97701</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -14116,22 +14166,22 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>district_id</t>
+          <t>ticket_id</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>route_date</t>
+          <t>execution_cycle</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>revision</t>
+          <t>appliance_id</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>previous_revision</t>
+          <t>office_id</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
@@ -14141,35 +14191,20 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>actor_id</t>
+          <t>movement</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>fingerprint</t>
+          <t>quantity</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>diff</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
-        <is>
-          <t>result</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>is_current</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>created_at</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
@@ -14183,7 +14218,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -14193,7 +14228,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>\N</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -14203,35 +14238,20 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>consume</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>93804b6a82cb845e7bf368040bd158224af7bfadb3a11d0a585f119745a97701</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>{}</t>
+          <t>2026-09-21T08:00:00+03:00</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -14314,113 +14334,6 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>ticket_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>execution_cycle</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>appliance_id</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>office_id</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>event_id</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>movement</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>quantity</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>created_at</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>consume</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>2026-09-21T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
           <t>worker_id</t>
         </is>
       </c>

</xml_diff>